<commit_message>
Switch SHAP to LHS+surrogate beeswarm; fix colorbar layout
tea_pareto_shap.py now Latin-hypercube samples N=128 points per frontier point
over the §4.7 driver ranges (128 real TEA calls), fits a gradient-boosted
surrogate (in-sample R2>=0.999, asserted), and runs TreeSHAP -> beeswarm.
Replaces the earlier single-instance exact-KernelSHAP bar/scatter. Colorbar
placed via constrained_layout (SA_RC autolayout fought it); figsize 9x4.5.
Log summary + history moved to _Tornado_Sensitivity.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgcoY62Dv9yGfFCEsMFckn
</commit_message>
<xml_diff>
--- a/Result/shap_ccs25_vs_nh325.xlsx
+++ b/Result/shap_ccs25_vs_nh325.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,17 +441,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>shap_usd_per_L</t>
+          <t>mean_abs_shap</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>base_mjsp</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>high_mjsp</t>
+          <t>mean_shap</t>
         </is>
       </c>
     </row>
@@ -467,13 +462,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.2585</v>
+        <v>0.3117</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.8716</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +476,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Co-product</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.4937</v>
+        <v>0.1032</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1.8716</v>
+        <v>-0.0014</v>
       </c>
     </row>
     <row r="4">
@@ -505,17 +494,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>Co-product</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.4783</v>
+        <v>0.0946</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.8716</v>
+        <v>-0.0002</v>
       </c>
     </row>
     <row r="5">
@@ -530,13 +516,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.3395</v>
+        <v>0.0584</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1.8716</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="6">
@@ -551,13 +534,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.1862</v>
+        <v>0.0201</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1.8716</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="7">
@@ -572,13 +552,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.1085</v>
+        <v>0.0102</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1.8716</v>
+        <v>-0.0003</v>
       </c>
     </row>
     <row r="8">
@@ -593,13 +570,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0518</v>
+        <v>0.0035</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9939</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.8716</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="9">
@@ -614,13 +588,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9439</v>
+        <v>0.2261</v>
       </c>
       <c r="D9" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E9" t="n">
-        <v>2.1936</v>
+        <v>-0.003</v>
       </c>
     </row>
     <row r="10">
@@ -635,13 +606,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5856</v>
+        <v>0.1245</v>
       </c>
       <c r="D10" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2.1936</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="11">
@@ -652,17 +620,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Co-product</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.4937</v>
+        <v>0.0998</v>
       </c>
       <c r="D11" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2.1936</v>
+        <v>-0.0004</v>
       </c>
     </row>
     <row r="12">
@@ -673,17 +638,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>Co-product</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4896</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2.1936</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="13">
@@ -698,13 +660,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.3581</v>
+        <v>0.0566</v>
       </c>
       <c r="D13" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2.1936</v>
+        <v>-0.0003</v>
       </c>
     </row>
     <row r="14">
@@ -719,13 +678,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.2284</v>
+        <v>0.0259</v>
       </c>
       <c r="D14" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E14" t="n">
-        <v>2.1936</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="15">
@@ -740,13 +696,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.0518</v>
+        <v>0.0042</v>
       </c>
       <c r="D15" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2.1936</v>
+        <v>0.0002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>